<commit_message>
added a new feature to the lottery game that allows players to select multiple numbers for their ticket. This enhancement increases the chances of winning and adds more excitement to the game. The user interface has been updated to accommodate the new multi-selection option, and the backend logic has been modified to handle multiple number selections during the ticket validation process. This update aims to provide a more engaging and enjoyable gaming experience for our users.
</commit_message>
<xml_diff>
--- a/megamillions_game.xlsx
+++ b/megamillions_game.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,56 +425,56 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J101"/>
+  <dimension ref="A1:J105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>GameName</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Day</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Year</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Num1</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Num2</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Num3</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Num4</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Num5</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>MegaBall</t>
         </is>
@@ -3866,6 +3878,142 @@
       </c>
       <c r="J101" t="n">
         <v>24</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Mega Millions</t>
+        </is>
+      </c>
+      <c r="B102" t="n">
+        <v>6</v>
+      </c>
+      <c r="C102" t="n">
+        <v>2</v>
+      </c>
+      <c r="D102" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E102" t="n">
+        <v>15</v>
+      </c>
+      <c r="F102" t="n">
+        <v>26</v>
+      </c>
+      <c r="G102" t="n">
+        <v>43</v>
+      </c>
+      <c r="H102" t="n">
+        <v>48</v>
+      </c>
+      <c r="I102" t="n">
+        <v>60</v>
+      </c>
+      <c r="J102" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Mega Millions</t>
+        </is>
+      </c>
+      <c r="B103" t="n">
+        <v>5</v>
+      </c>
+      <c r="C103" t="n">
+        <v>29</v>
+      </c>
+      <c r="D103" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E103" t="n">
+        <v>19</v>
+      </c>
+      <c r="F103" t="n">
+        <v>24</v>
+      </c>
+      <c r="G103" t="n">
+        <v>47</v>
+      </c>
+      <c r="H103" t="n">
+        <v>59</v>
+      </c>
+      <c r="I103" t="n">
+        <v>65</v>
+      </c>
+      <c r="J103" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Mega Millions</t>
+        </is>
+      </c>
+      <c r="B104" t="n">
+        <v>5</v>
+      </c>
+      <c r="C104" t="n">
+        <v>26</v>
+      </c>
+      <c r="D104" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E104" t="n">
+        <v>1</v>
+      </c>
+      <c r="F104" t="n">
+        <v>5</v>
+      </c>
+      <c r="G104" t="n">
+        <v>49</v>
+      </c>
+      <c r="H104" t="n">
+        <v>51</v>
+      </c>
+      <c r="I104" t="n">
+        <v>59</v>
+      </c>
+      <c r="J104" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Mega Millions</t>
+        </is>
+      </c>
+      <c r="B105" t="n">
+        <v>6</v>
+      </c>
+      <c r="C105" t="n">
+        <v>5</v>
+      </c>
+      <c r="D105" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E105" t="n">
+        <v>13</v>
+      </c>
+      <c r="F105" t="n">
+        <v>30</v>
+      </c>
+      <c r="G105" t="n">
+        <v>50</v>
+      </c>
+      <c r="H105" t="n">
+        <v>52</v>
+      </c>
+      <c r="I105" t="n">
+        <v>66</v>
+      </c>
+      <c r="J105" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>